<commit_message>
chore: update schedules 2026-09-19
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,17 +498,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>026D6</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>23-Sep-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>026D6</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -597,22 +597,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>026E5</t>
+          <t>02640</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -649,22 +649,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>02640</t>
+          <t>026E5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>21-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -986,17 +986,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,17 +1013,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1100,24 +1100,24 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>19-Sep-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,49 +1142,49 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>26-Sep-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>026E3</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1194,49 +1194,49 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>026E5</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>02-Jan-2027</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14-Oct-2026</t>
+          <t>19-Sep-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>26-Sep-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DAMMAM</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,42 +1377,42 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>27-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGLX</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ESL KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>026E5</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>23-Oct-2026</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>KMT TBN</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>02643</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>15-Nov-2026</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>14-Oct-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,86 +1506,86 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-18 03:25 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>18-Sep-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>KMT TBN</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>00639</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1610,69 +1610,69 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>19-Sep-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>00438</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1684,47 +1684,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>19-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>00438</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>24-Sep-2026</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>KMTC DAMMAM</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>026E3</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1736,47 +1736,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23-Sep-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>KMTC DAMMAM</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00640</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>27-Sep-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1788,47 +1788,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>23-Sep-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>026E5</t>
+          <t>00439</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>26-Sep-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1840,47 +1840,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>23-Sep-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00439</t>
+          <t>026E5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>26-Sep-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1892,47 +1892,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>23-Sep-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>00639</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>27-Sep-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1944,47 +1944,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00641</t>
+          <t>026E5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -1996,47 +1996,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>27-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>HUAXIN968</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>00640</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>16-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>BHUDTHI BHUM</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>026E6</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2063,32 +2063,32 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>00441</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>05-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>03-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2167,12 +2167,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>00641</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,17 +2182,17 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>KMT TBN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2234,17 +2234,17 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2271,32 +2271,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>00441</t>
+          <t>00642</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>05-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>06-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2323,32 +2323,32 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,12 +2360,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>00643</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,37 +2464,37 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01099</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2504,24 +2504,24 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15-Sep-2026</t>
+          <t>14-Oct-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2531,64 +2531,64 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2636E</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,34 +2598,34 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>18-Oct-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2635,49 +2635,49 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2637E</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>29-Sep-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>25-Sep-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2692,79 +2692,79 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01062</t>
+          <t>01201</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>03-Oct-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>26-Sep-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01091</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>29-Sep-2026</t>
+          <t>15-Sep-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2638E</t>
+          <t>2636E</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>06-Oct-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2828,47 +2828,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>30-Sep-2026</t>
+          <t>14-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01092</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>08-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>03-Oct-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2895,12 +2895,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ZHONG YI RUN HAI</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01064</t>
+          <t>2637E</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,17 +2910,17 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-09-18 03:26 UTC</t>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>
@@ -2937,42 +2937,302 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>01062</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>03-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>26-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>01091</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>04-Oct-2026</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ZHONG YI RUN HAI</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2638E</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>06-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>30-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>01092</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>08-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>03-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>01064</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>04-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
         <is>
           <t>01093</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>12-Oct-2026</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-09-18 03:26 UTC</t>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-09-19 03:22 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>